<commit_message>
Gencon 2026 Promo cards added
</commit_message>
<xml_diff>
--- a/cards_template_excel.xlsx
+++ b/cards_template_excel.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84240D90-7A1C-496C-93C7-AB221100613E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFDB243B-1551-4B03-A17D-5EE98C1FE889}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4951" uniqueCount="2511">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4974" uniqueCount="2523">
   <si>
     <t>Name</t>
   </si>
@@ -7548,6 +7548,42 @@
   </si>
   <si>
     <t>zoe.jpg</t>
+  </si>
+  <si>
+    <t>Starchy</t>
+  </si>
+  <si>
+    <t>starchy.jpg</t>
+  </si>
+  <si>
+    <t>Once per turn, you may remove target Creature in a discard pile from the game and draw a card.</t>
+  </si>
+  <si>
+    <t>Sweet Delicious Meats</t>
+  </si>
+  <si>
+    <t>Target player heals 1 HP for each card that is removed from the game.</t>
+  </si>
+  <si>
+    <t>sweet_delicious_meats.jpg</t>
+  </si>
+  <si>
+    <t>Probably Too Many Unicorns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When this Creature enters play, reveal the bottom 4 cards of target player's deck. Put all Creatures revealed into their discard pile and the rest on top of their deck in any order. If this Creature is defeated, put it on the bottom of your deck. </t>
+  </si>
+  <si>
+    <t>probably_too_many_unicorns.jpg</t>
+  </si>
+  <si>
+    <t>Time Drake</t>
+  </si>
+  <si>
+    <t>time_drake.jpg</t>
+  </si>
+  <si>
+    <t>When Time Drake enters play, reveal the top 5 cards of target player's deck. Put all Creatures revealed into their discard pile and return the rest to the top of their deck in any order. Add an :attack_token: to Time Drake for each Creature put into a discard pile this way.</t>
   </si>
 </sst>
 </file>
@@ -7889,11 +7925,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I836"/>
+  <dimension ref="A1:I840"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="45.6640625" customWidth="1"/>
+    <col min="1" max="1" width="28.109375" customWidth="1"/>
     <col min="4" max="4" width="82.5546875" customWidth="1"/>
+    <col min="6" max="6" width="27.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
@@ -30380,6 +30417,104 @@
         <v>11</v>
       </c>
     </row>
+    <row r="837" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A837" t="s">
+        <v>2511</v>
+      </c>
+      <c r="B837" t="s">
+        <v>10</v>
+      </c>
+      <c r="D837" t="s">
+        <v>2513</v>
+      </c>
+      <c r="E837" t="s">
+        <v>1505</v>
+      </c>
+      <c r="F837" t="s">
+        <v>2512</v>
+      </c>
+    </row>
+    <row r="838" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A838" t="s">
+        <v>2514</v>
+      </c>
+      <c r="B838" t="s">
+        <v>112</v>
+      </c>
+      <c r="C838" t="s">
+        <v>168</v>
+      </c>
+      <c r="D838" t="s">
+        <v>2515</v>
+      </c>
+      <c r="E838" t="s">
+        <v>1505</v>
+      </c>
+      <c r="F838" t="s">
+        <v>2516</v>
+      </c>
+      <c r="G838">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="839" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A839" t="s">
+        <v>2517</v>
+      </c>
+      <c r="B839" t="s">
+        <v>18</v>
+      </c>
+      <c r="C839" t="s">
+        <v>168</v>
+      </c>
+      <c r="D839" t="s">
+        <v>2518</v>
+      </c>
+      <c r="E839" t="s">
+        <v>1505</v>
+      </c>
+      <c r="F839" t="s">
+        <v>2519</v>
+      </c>
+      <c r="G839">
+        <v>1</v>
+      </c>
+      <c r="H839">
+        <v>1</v>
+      </c>
+      <c r="I839">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="840" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A840" t="s">
+        <v>2520</v>
+      </c>
+      <c r="B840" t="s">
+        <v>18</v>
+      </c>
+      <c r="C840" t="s">
+        <v>168</v>
+      </c>
+      <c r="D840" t="s">
+        <v>2522</v>
+      </c>
+      <c r="E840" t="s">
+        <v>1505</v>
+      </c>
+      <c r="F840" t="s">
+        <v>2521</v>
+      </c>
+      <c r="G840">
+        <v>2</v>
+      </c>
+      <c r="H840">
+        <v>0</v>
+      </c>
+      <c r="I840">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Me-Mow and Flame Princess
</commit_message>
<xml_diff>
--- a/cards_template_excel.xlsx
+++ b/cards_template_excel.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFDB243B-1551-4B03-A17D-5EE98C1FE889}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0DC89CE-6B1B-4BF0-8024-65333E4FBCA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4974" uniqueCount="2523">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4984" uniqueCount="2528">
   <si>
     <t>Name</t>
   </si>
@@ -7584,6 +7584,21 @@
   </si>
   <si>
     <t>When Time Drake enters play, reveal the top 5 cards of target player's deck. Put all Creatures revealed into their discard pile and return the rest to the top of their deck in any order. Add an :attack_token: to Time Drake for each Creature put into a discard pile this way.</t>
+  </si>
+  <si>
+    <t>Me-Mow</t>
+  </si>
+  <si>
+    <t>During each of your turns, the first time you deal exactly 1 damage to an opposing Creature, remove the bottom card of target opponent's deck from the game. (Limit: Once per opposing Creature per turn.)</t>
+  </si>
+  <si>
+    <t>me-mow.jpg</t>
+  </si>
+  <si>
+    <t>Flame Princess Promo</t>
+  </si>
+  <si>
+    <t>flame_princess_promo.jpg</t>
   </si>
 </sst>
 </file>
@@ -7925,7 +7940,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I840"/>
+  <dimension ref="A1:I842"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28.109375" customWidth="1"/>
@@ -30515,6 +30530,40 @@
         <v>8</v>
       </c>
     </row>
+    <row r="841" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A841" t="s">
+        <v>2523</v>
+      </c>
+      <c r="B841" t="s">
+        <v>10</v>
+      </c>
+      <c r="D841" t="s">
+        <v>2524</v>
+      </c>
+      <c r="E841" t="s">
+        <v>1505</v>
+      </c>
+      <c r="F841" t="s">
+        <v>2525</v>
+      </c>
+    </row>
+    <row r="842" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A842" t="s">
+        <v>2526</v>
+      </c>
+      <c r="B842" t="s">
+        <v>10</v>
+      </c>
+      <c r="D842" t="s">
+        <v>1733</v>
+      </c>
+      <c r="E842" t="s">
+        <v>1505</v>
+      </c>
+      <c r="F842" t="s">
+        <v>2527</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>